<commit_message>
"Update for the day."
</commit_message>
<xml_diff>
--- a/Output_Data/Integrated_Values/Right_Leg/ICC_By_Mean/Integrated_Values_Edited.xlsx
+++ b/Output_Data/Integrated_Values/Right_Leg/ICC_By_Mean/Integrated_Values_Edited.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24729"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,14 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Customer\Projects\MultiCam_Study\Output_Data\Integrated_Values\Right_Leg\ICC_By_Mean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{C0D30DF1-D0EF-4FC5-ACAB-B8D1E24E174C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D776BEC-4F42-4910-8363-FA44B78AB5EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4932" yWindow="720" windowWidth="17280" windowHeight="8880"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Integrated_Values" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -88,7 +100,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -406,7 +418,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -521,6 +533,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -566,8 +593,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -922,484 +950,487 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="16384" width="8.88671875" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>0.95362426857228</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="1">
         <v>0.94406818043962004</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="1">
         <v>0.85727925538421001</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="1">
         <f>AVERAGE(C2:E2)</f>
         <v>0.91832390146537002</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="1">
         <v>0.45999316802830897</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="1">
         <v>0.58875647396180397</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="1">
         <v>0.67583713535790801</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="1">
         <f>AVERAGE(G2:I2)</f>
         <v>0.57486225911600697</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>0.84365354448144303</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="1">
         <v>0.82354731475353304</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
         <v>0.51946352098587301</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="1">
         <f t="shared" ref="F3:F13" si="0">AVERAGE(C3:E3)</f>
         <v>0.72888812674028303</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="1">
         <v>0.47290973449707502</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="1">
         <v>0.51308023058888597</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="1">
         <v>0.56491012105898197</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="1">
         <f t="shared" ref="J3:J13" si="1">AVERAGE(G3:I3)</f>
         <v>0.51696669538164763</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>0.92021595998647898</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>0.90613293794530103</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="1">
         <v>0.89662404620698399</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="1">
         <f t="shared" si="0"/>
         <v>0.90765764804625471</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="1">
         <v>0.62054767646454201</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="1">
         <v>0.70774478371716498</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="1">
         <v>0.65783422750369203</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="1">
         <f t="shared" si="1"/>
         <v>0.66204222922846634</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.95314285309852997</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.94109284948821503</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.90294354134133303</v>
+      </c>
+      <c r="F5" s="1">
+        <f>AVERAGE(C5:E5)</f>
+        <v>0.93239308130935938</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0.58165407561457805</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0.67445562545904902</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0.77205333625658501</v>
+      </c>
+      <c r="J5" s="1">
+        <f>AVERAGE(G5:I5)</f>
+        <v>0.67605434577673729</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.97301069351478198</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.96656749769023298</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.95271785950187204</v>
+      </c>
+      <c r="F6" s="1">
+        <f>AVERAGE(C6:E6)</f>
+        <v>0.96409868356896233</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0.309181429169886</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0.36013119292935802</v>
+      </c>
+      <c r="I6" s="1">
+        <v>0.32523198331665998</v>
+      </c>
+      <c r="J6" s="1">
+        <f>AVERAGE(G6:I6)</f>
+        <v>0.33151486847196798</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.79155385103439801</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.808189397090738</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.72998696616467396</v>
+      </c>
+      <c r="F7" s="1">
+        <f>AVERAGE(C7:E7)</f>
+        <v>0.77657673809660333</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0.60263080490956999</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0.63549934274671305</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0.74535913635509798</v>
+      </c>
+      <c r="J7" s="1">
+        <f>AVERAGE(G7:I7)</f>
+        <v>0.66116309467046042</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C5">
+      <c r="C8" s="1">
         <v>0.93119484058216895</v>
       </c>
-      <c r="D5">
+      <c r="D8" s="1">
         <v>0.89144162272856897</v>
       </c>
-      <c r="E5">
+      <c r="E8" s="1">
         <v>0.91668942620721705</v>
       </c>
-      <c r="F5">
+      <c r="F8" s="1">
         <f t="shared" si="0"/>
         <v>0.91310862983931829</v>
       </c>
-      <c r="G5">
+      <c r="G8" s="1">
         <v>0.65836540398660504</v>
       </c>
-      <c r="H5">
+      <c r="H8" s="1">
         <v>0.77426753730060105</v>
       </c>
-      <c r="I5">
+      <c r="I8" s="1">
         <v>0.74692503772915297</v>
       </c>
-      <c r="J5">
+      <c r="J8" s="1">
         <f t="shared" si="1"/>
         <v>0.72651932633878635</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C6">
+      <c r="C9" s="1">
         <v>0.94435307228534404</v>
       </c>
-      <c r="D6">
+      <c r="D9" s="1">
         <v>0.938040926584086</v>
       </c>
-      <c r="E6">
+      <c r="E9" s="1">
         <v>0.86109768133417797</v>
       </c>
-      <c r="F6">
+      <c r="F9" s="1">
         <f t="shared" si="0"/>
         <v>0.91449722673453593</v>
       </c>
-      <c r="G6">
+      <c r="G9" s="1">
         <v>0.43811859756583399</v>
       </c>
-      <c r="H6">
+      <c r="H9" s="1">
         <v>0.50485805013347096</v>
       </c>
-      <c r="I6">
+      <c r="I9" s="1">
         <v>0.57444915340556202</v>
       </c>
-      <c r="J6">
+      <c r="J9" s="1">
         <f t="shared" si="1"/>
         <v>0.50580860036828901</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C7">
+      <c r="C10" s="1">
         <v>0.94705865778521103</v>
       </c>
-      <c r="D7">
+      <c r="D10" s="1">
         <v>0.91544455985603301</v>
       </c>
-      <c r="E7">
+      <c r="E10" s="1">
         <v>0.91982582474683605</v>
       </c>
-      <c r="F7">
+      <c r="F10" s="1">
         <f t="shared" si="0"/>
         <v>0.92744301412936003</v>
       </c>
-      <c r="G7">
+      <c r="G10" s="1">
         <v>0.47990684634103697</v>
       </c>
-      <c r="H7">
+      <c r="H10" s="1">
         <v>0.56026629232333303</v>
       </c>
-      <c r="I7">
+      <c r="I10" s="1">
         <v>0.52221158996524797</v>
       </c>
-      <c r="J7">
+      <c r="J10" s="1">
         <f t="shared" si="1"/>
         <v>0.52079490954320595</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8">
-        <v>0.95314285309852997</v>
-      </c>
-      <c r="D8">
-        <v>0.94109284948821503</v>
-      </c>
-      <c r="E8">
-        <v>0.90294354134133303</v>
-      </c>
-      <c r="F8">
-        <f t="shared" si="0"/>
-        <v>0.93239308130935938</v>
-      </c>
-      <c r="G8">
-        <v>0.58165407561457805</v>
-      </c>
-      <c r="H8">
-        <v>0.67445562545904902</v>
-      </c>
-      <c r="I8">
-        <v>0.77205333625658501</v>
-      </c>
-      <c r="J8">
-        <f t="shared" si="1"/>
-        <v>0.67605434577673729</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9">
-        <v>0.97301069351478198</v>
-      </c>
-      <c r="D9">
-        <v>0.96656749769023298</v>
-      </c>
-      <c r="E9">
-        <v>0.95271785950187204</v>
-      </c>
-      <c r="F9">
-        <f t="shared" si="0"/>
-        <v>0.96409868356896233</v>
-      </c>
-      <c r="G9">
-        <v>0.309181429169886</v>
-      </c>
-      <c r="H9">
-        <v>0.36013119292935802</v>
-      </c>
-      <c r="I9">
-        <v>0.32523198331665998</v>
-      </c>
-      <c r="J9">
-        <f t="shared" si="1"/>
-        <v>0.33151486847196798</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10">
-        <v>0.79155385103439801</v>
-      </c>
-      <c r="D10">
-        <v>0.808189397090738</v>
-      </c>
-      <c r="E10">
-        <v>0.72998696616467396</v>
-      </c>
-      <c r="F10">
-        <f t="shared" si="0"/>
-        <v>0.77657673809660333</v>
-      </c>
-      <c r="G10">
-        <v>0.60263080490956999</v>
-      </c>
-      <c r="H10">
-        <v>0.63549934274671305</v>
-      </c>
-      <c r="I10">
-        <v>0.74535913635509798</v>
-      </c>
-      <c r="J10">
-        <f t="shared" si="1"/>
-        <v>0.66116309467046042</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11">
+      <c r="C11" s="1">
         <v>0.86426805264417805</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="1">
         <v>0.75323932282029205</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="1">
         <v>0.79466028344027095</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="1">
         <f t="shared" si="0"/>
         <v>0.8040558863015802</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="1">
         <v>0.46860313895865502</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="1">
         <v>0.55372607517377803</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="1">
         <v>0.51347988670706601</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="1">
         <f t="shared" si="1"/>
         <v>0.51193636694649969</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="1">
         <v>0.91393929034786603</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="1">
         <v>0.92369775667860199</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="1">
         <v>0.89857516983225105</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="1">
         <f t="shared" si="0"/>
         <v>0.91207073895290636</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="1">
         <v>0.39699967262458502</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="1">
         <v>0.40542284583687499</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="1">
         <v>0.498319800118385</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="1">
         <f t="shared" si="1"/>
         <v>0.43358077285994834</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="1">
         <v>0.98653463523683305</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="1">
         <v>0.95561104992758605</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="1">
         <v>0.96255957520575597</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="1">
         <f t="shared" si="0"/>
         <v>0.96823508679005832</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="1">
         <v>0.28505306740078701</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="1">
         <v>0.43202156244204298</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="1">
         <v>0.42336560892949798</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="1">
         <f t="shared" si="1"/>
         <v>0.38014674625744266</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="1">
         <f>AVERAGE(C2:E13)</f>
-        <v>0.88894573016454936</v>
+        <v>0.8889457301645497</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="1">
         <f>_xlfn.STDEV.S(C2:E13)</f>
-        <v>8.9594144076058188E-2</v>
+        <v>8.9594144076058174E-2</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="1">
         <f>AVERAGE(H2:J13)</f>
-        <v>0.56198881234101039</v>
+        <v>0.56198881234101028</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="1">
         <f>_xlfn.STDEV.S(H2:J13)</f>
-        <v>0.12678781704201555</v>
+        <v>0.12678781704201636</v>
       </c>
     </row>
   </sheetData>

</xml_diff>